<commit_message>
Compute footprint area geodesically instead of parsing description text
Google Earth's own Area measurement (geodesic, WGS84 ellipsoid) matches
the description text closely for OSM-sourced footprints, confirming the
polygon coordinates are the reliable ground truth. Switched from parsing
"X m²" out of the description string to computing polygon area directly
via pyproj.Geod, which also fills in area for the 29 "Client existant"
placemarks that have no description text at all.
</commit_message>
<xml_diff>
--- a/BMR_prospection.xlsx
+++ b/BMR_prospection.xlsx
@@ -450,7 +450,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,9 +521,17 @@
           <t>G5J 2G3</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
+        <v>1307</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>14066</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -551,9 +559,17 @@
           <t>J1A1N2</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="n">
+        <v>1339</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>14408</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -581,9 +597,17 @@
           <t>J0B 1L0</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>9730</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -611,9 +635,17 @@
           <t>G0N 1E0</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="n">
+        <v>1007</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>10838</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -641,9 +673,17 @@
           <t>J0T 1G0</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>3661</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -671,9 +711,17 @@
           <t>J0T 1S0</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="n">
+        <v>339</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>3648</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -701,9 +749,17 @@
           <t>G0S 1P0</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="n">
+        <v>1053</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>11331</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -731,9 +787,17 @@
           <t>G4T 3E6</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="n">
+        <v>3110</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>33477</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -761,9 +825,17 @@
           <t>G4W 1A9</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
+        <v>508</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>5469</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -791,9 +863,17 @@
           <t>G4W 1A5</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="n">
+        <v>1003</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>10799</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -821,9 +901,17 @@
           <t>G5H 3Y1</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="n">
+        <v>1372</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>14765</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -851,9 +939,17 @@
           <t>J0W 1R0</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="n">
+        <v>1077</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>11596</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -881,9 +977,17 @@
           <t>G5L 2T2</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>6261</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>67397</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -911,9 +1015,17 @@
           <t>G3L 2Y6</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>1458</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>15698</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -941,9 +1053,17 @@
           <t>G0L 2G0</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>1474</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>15865</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -971,9 +1091,17 @@
           <t>G0L 2J0</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>1697</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>18271</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1001,9 +1129,17 @@
           <t>G0N 1N0</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>1106</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>11900</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1031,9 +1167,17 @@
           <t>J0B 2V0</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>997</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>10736</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1061,9 +1205,17 @@
           <t>J0B 2T0</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>746</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>8033</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1091,9 +1243,17 @@
           <t>J2T 3G4</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>3403</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>36630</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1121,9 +1281,17 @@
           <t>G0N 1J0</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>776</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>8348</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1151,9 +1319,17 @@
           <t>G0L 3M0</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
+        <v>1172</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>12610</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1181,9 +1357,17 @@
           <t>G0R 3J0</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>2174</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>23403</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1211,9 +1395,17 @@
           <t>J0C 1M0</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>499</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>5368</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1241,9 +1433,17 @@
           <t>J0K 2T0</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>1290</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>13888</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1271,9 +1471,17 @@
           <t>G0L 4K0</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>1112</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>11973</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1301,9 +1509,17 @@
           <t>J1T 3Z1</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>1945</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>20932</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1331,9 +1547,17 @@
           <t>J0B 3J0</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="n">
+        <v>1285</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>13826</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1361,9 +1585,17 @@
           <t>J0A 1N0</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>1567</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>16868</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Manuel (client)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1392,10 +1624,10 @@
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>706</v>
+        <v>1181</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>7601</v>
+        <v>12712</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
@@ -1430,10 +1662,10 @@
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>616</v>
+        <v>690</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>6632</v>
+        <v>7424</v>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
@@ -1506,10 +1738,10 @@
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>723</v>
+        <v>767</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>7777</v>
+        <v>8257</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
@@ -1544,10 +1776,10 @@
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>909</v>
+        <v>952</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
@@ -1582,10 +1814,10 @@
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>392</v>
+        <v>760</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>4223</v>
+        <v>8185</v>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
@@ -1620,10 +1852,10 @@
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>1537</v>
+        <v>2306</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>16548</v>
+        <v>24820</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
@@ -1658,10 +1890,10 @@
         </is>
       </c>
       <c r="F38" s="3" t="n">
-        <v>1146</v>
+        <v>524</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>12340</v>
+        <v>5638</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
@@ -1696,10 +1928,10 @@
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1160</v>
+        <v>301</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>12484</v>
+        <v>3235</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
@@ -1734,10 +1966,10 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>317</v>
+        <v>906</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>3415</v>
+        <v>9751</v>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
@@ -1772,10 +2004,10 @@
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>119</v>
+        <v>261</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>1279</v>
+        <v>2807</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
@@ -1809,8 +2041,12 @@
           <t>G0A 1N0</t>
         </is>
       </c>
-      <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
+      <c r="F42" s="3" t="n">
+        <v>2526</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>27193</v>
+      </c>
       <c r="H42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1840,10 +2076,10 @@
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>774</v>
+        <v>1169</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>8328</v>
+        <v>12578</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
@@ -1878,10 +2114,10 @@
         </is>
       </c>
       <c r="F44" s="3" t="n">
-        <v>169</v>
+        <v>2022</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>1819</v>
+        <v>21762</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
@@ -1916,10 +2152,10 @@
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>1165</v>
+        <v>1068</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>12538</v>
+        <v>11492</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
@@ -1992,10 +2228,10 @@
         </is>
       </c>
       <c r="F47" s="3" t="n">
-        <v>1189</v>
+        <v>1235</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>12799</v>
+        <v>13290</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
@@ -2144,10 +2380,10 @@
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>1129</v>
+        <v>1116</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>12154</v>
+        <v>12007</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
@@ -2182,10 +2418,10 @@
         </is>
       </c>
       <c r="F52" s="3" t="n">
-        <v>719</v>
+        <v>876</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>7742</v>
+        <v>9425</v>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
@@ -2220,10 +2456,10 @@
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>6246</v>
+        <v>1114</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>67232</v>
+        <v>11992</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
@@ -2258,10 +2494,10 @@
         </is>
       </c>
       <c r="F54" s="3" t="n">
-        <v>751</v>
+        <v>453</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>8087</v>
+        <v>4881</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
@@ -2334,10 +2570,10 @@
         </is>
       </c>
       <c r="F56" s="3" t="n">
-        <v>1092</v>
+        <v>1098</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>11750</v>
+        <v>11822</v>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
@@ -2372,10 +2608,10 @@
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>192</v>
+        <v>863</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>2064</v>
+        <v>9289</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
@@ -2410,10 +2646,10 @@
         </is>
       </c>
       <c r="F58" s="3" t="n">
-        <v>1462</v>
+        <v>1612</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>15742</v>
+        <v>17350</v>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
@@ -2448,10 +2684,10 @@
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>2093</v>
+        <v>712</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>22533</v>
+        <v>7663</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
@@ -2524,10 +2760,10 @@
         </is>
       </c>
       <c r="F61" s="3" t="n">
-        <v>987</v>
+        <v>943</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>10623</v>
+        <v>10148</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
@@ -2676,10 +2912,10 @@
         </is>
       </c>
       <c r="F65" s="3" t="n">
-        <v>3647</v>
+        <v>2966</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>39252</v>
+        <v>31927</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -2714,10 +2950,10 @@
         </is>
       </c>
       <c r="F66" s="3" t="n">
-        <v>700</v>
+        <v>390</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>7537</v>
+        <v>4201</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
@@ -2752,10 +2988,10 @@
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>312</v>
+        <v>294</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>3355</v>
+        <v>3167</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -2828,10 +3064,10 @@
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>105</v>
+        <v>1267</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>1130</v>
+        <v>13643</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
@@ -2941,8 +3177,12 @@
           <t>G0W 1C0</t>
         </is>
       </c>
-      <c r="F72" s="3" t="n"/>
-      <c r="G72" s="3" t="n"/>
+      <c r="F72" s="3" t="n">
+        <v>802</v>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>8638</v>
+      </c>
       <c r="H72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
@@ -2972,10 +3212,10 @@
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>406</v>
+        <v>627</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>4372</v>
+        <v>6749</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
@@ -3010,10 +3250,10 @@
         </is>
       </c>
       <c r="F74" s="3" t="n">
-        <v>1083</v>
+        <v>759</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>11657</v>
+        <v>8167</v>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
@@ -3047,8 +3287,12 @@
           <t>G5V 3A6</t>
         </is>
       </c>
-      <c r="F75" s="3" t="n"/>
-      <c r="G75" s="3" t="n"/>
+      <c r="F75" s="3" t="n">
+        <v>2424</v>
+      </c>
+      <c r="G75" s="3" t="n">
+        <v>26094</v>
+      </c>
       <c r="H75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
@@ -3078,10 +3322,10 @@
         </is>
       </c>
       <c r="F76" s="3" t="n">
-        <v>2516</v>
+        <v>1258</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>27079</v>
+        <v>13539</v>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
@@ -3116,10 +3360,10 @@
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>552</v>
+        <v>101</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>5942</v>
+        <v>1085</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
@@ -3154,10 +3398,10 @@
         </is>
       </c>
       <c r="F78" s="3" t="n">
-        <v>523</v>
+        <v>243</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>5629</v>
+        <v>2620</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
@@ -3191,8 +3435,12 @@
           <t>H1W 1R8</t>
         </is>
       </c>
-      <c r="F79" s="3" t="n"/>
-      <c r="G79" s="3" t="n"/>
+      <c r="F79" s="3" t="n">
+        <v>225</v>
+      </c>
+      <c r="G79" s="3" t="n">
+        <v>2424</v>
+      </c>
       <c r="H79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
@@ -3222,10 +3470,10 @@
         </is>
       </c>
       <c r="F80" s="3" t="n">
-        <v>1036</v>
+        <v>834</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>11148</v>
+        <v>8975</v>
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
@@ -3260,10 +3508,10 @@
         </is>
       </c>
       <c r="F81" s="3" t="n">
-        <v>1631</v>
+        <v>193</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>17560</v>
+        <v>2076</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
@@ -3298,10 +3546,10 @@
         </is>
       </c>
       <c r="F82" s="3" t="n">
-        <v>983</v>
+        <v>2383</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>10585</v>
+        <v>25646</v>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
@@ -3336,10 +3584,10 @@
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>125</v>
+        <v>1552</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>1346</v>
+        <v>16709</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
@@ -3412,10 +3660,10 @@
         </is>
       </c>
       <c r="F85" s="3" t="n">
-        <v>109</v>
+        <v>404</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>1172</v>
+        <v>4353</v>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
@@ -3450,10 +3698,10 @@
         </is>
       </c>
       <c r="F86" s="3" t="n">
-        <v>869</v>
+        <v>730</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>9350</v>
+        <v>7856</v>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
@@ -3488,10 +3736,10 @@
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>9755</v>
+        <v>9697</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
@@ -3526,10 +3774,10 @@
         </is>
       </c>
       <c r="F88" s="3" t="n">
-        <v>456</v>
+        <v>484</v>
       </c>
       <c r="G88" s="3" t="n">
-        <v>4913</v>
+        <v>5209</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
@@ -3602,10 +3850,10 @@
         </is>
       </c>
       <c r="F90" s="3" t="n">
-        <v>1642</v>
+        <v>1170</v>
       </c>
       <c r="G90" s="3" t="n">
-        <v>17671</v>
+        <v>12597</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
@@ -3678,10 +3926,10 @@
         </is>
       </c>
       <c r="F92" s="3" t="n">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>2389</v>
+        <v>2526</v>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
@@ -3716,10 +3964,10 @@
         </is>
       </c>
       <c r="F93" s="3" t="n">
-        <v>993</v>
+        <v>818</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>10685</v>
+        <v>8800</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
@@ -3754,10 +4002,10 @@
         </is>
       </c>
       <c r="F94" s="3" t="n">
-        <v>273</v>
+        <v>342</v>
       </c>
       <c r="G94" s="3" t="n">
-        <v>2944</v>
+        <v>3680</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
@@ -3792,10 +4040,10 @@
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>3168</v>
+        <v>1487</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>34095</v>
+        <v>16009</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
@@ -3868,10 +4116,10 @@
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>601</v>
+        <v>642</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>6474</v>
+        <v>6913</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
@@ -3906,10 +4154,10 @@
         </is>
       </c>
       <c r="F98" s="3" t="n">
-        <v>194</v>
+        <v>815</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>2094</v>
+        <v>8776</v>
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
@@ -3944,10 +4192,10 @@
         </is>
       </c>
       <c r="F99" s="3" t="n">
-        <v>718</v>
+        <v>768</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>7731</v>
+        <v>8271</v>
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
@@ -3982,10 +4230,10 @@
         </is>
       </c>
       <c r="F100" s="3" t="n">
-        <v>740</v>
+        <v>850</v>
       </c>
       <c r="G100" s="3" t="n">
-        <v>7961</v>
+        <v>9154</v>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
@@ -4057,8 +4305,12 @@
           <t>G0M 1J0</t>
         </is>
       </c>
-      <c r="F102" s="3" t="n"/>
-      <c r="G102" s="3" t="n"/>
+      <c r="F102" s="3" t="n">
+        <v>716</v>
+      </c>
+      <c r="G102" s="3" t="n">
+        <v>7705</v>
+      </c>
       <c r="H102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
@@ -4088,10 +4340,10 @@
         </is>
       </c>
       <c r="F103" s="3" t="n">
-        <v>896</v>
+        <v>1410</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>9647</v>
+        <v>15180</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
@@ -4126,10 +4378,10 @@
         </is>
       </c>
       <c r="F104" s="3" t="n">
-        <v>48</v>
+        <v>503</v>
       </c>
       <c r="G104" s="3" t="n">
-        <v>513</v>
+        <v>5410</v>
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
@@ -4202,10 +4454,10 @@
         </is>
       </c>
       <c r="F106" s="3" t="n">
-        <v>3114</v>
+        <v>3400</v>
       </c>
       <c r="G106" s="3" t="n">
-        <v>33524</v>
+        <v>36602</v>
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
@@ -4240,10 +4492,10 @@
         </is>
       </c>
       <c r="F107" s="3" t="n">
-        <v>880</v>
+        <v>166</v>
       </c>
       <c r="G107" s="3" t="n">
-        <v>9471</v>
+        <v>1789</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
@@ -4278,10 +4530,10 @@
         </is>
       </c>
       <c r="F108" s="3" t="n">
-        <v>2775</v>
+        <v>2793</v>
       </c>
       <c r="G108" s="3" t="n">
-        <v>29871</v>
+        <v>30061</v>
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
@@ -4392,10 +4644,10 @@
         </is>
       </c>
       <c r="F111" s="3" t="n">
-        <v>604</v>
+        <v>631</v>
       </c>
       <c r="G111" s="3" t="n">
-        <v>6501</v>
+        <v>6795</v>
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
@@ -4430,10 +4682,10 @@
         </is>
       </c>
       <c r="F112" s="3" t="n">
-        <v>827</v>
+        <v>1812</v>
       </c>
       <c r="G112" s="3" t="n">
-        <v>8900</v>
+        <v>19505</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
@@ -4468,10 +4720,10 @@
         </is>
       </c>
       <c r="F113" s="3" t="n">
-        <v>666</v>
+        <v>762</v>
       </c>
       <c r="G113" s="3" t="n">
-        <v>7172</v>
+        <v>8204</v>
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
@@ -4506,10 +4758,10 @@
         </is>
       </c>
       <c r="F114" s="3" t="n">
-        <v>1084</v>
+        <v>808</v>
       </c>
       <c r="G114" s="3" t="n">
-        <v>11669</v>
+        <v>8694</v>
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
@@ -4544,10 +4796,10 @@
         </is>
       </c>
       <c r="F115" s="3" t="n">
-        <v>488</v>
+        <v>397</v>
       </c>
       <c r="G115" s="3" t="n">
-        <v>5255</v>
+        <v>4272</v>
       </c>
       <c r="H115" s="3" t="inlineStr">
         <is>
@@ -4582,10 +4834,10 @@
         </is>
       </c>
       <c r="F116" s="3" t="n">
-        <v>137</v>
+        <v>1547</v>
       </c>
       <c r="G116" s="3" t="n">
-        <v>1479</v>
+        <v>16653</v>
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
@@ -4620,10 +4872,10 @@
         </is>
       </c>
       <c r="F117" s="3" t="n">
-        <v>913</v>
+        <v>525</v>
       </c>
       <c r="G117" s="3" t="n">
-        <v>9827</v>
+        <v>5654</v>
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
@@ -4658,10 +4910,10 @@
         </is>
       </c>
       <c r="F118" s="3" t="n">
-        <v>399</v>
+        <v>538</v>
       </c>
       <c r="G118" s="3" t="n">
-        <v>4299</v>
+        <v>5794</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
@@ -4696,10 +4948,10 @@
         </is>
       </c>
       <c r="F119" s="3" t="n">
-        <v>982</v>
+        <v>977</v>
       </c>
       <c r="G119" s="3" t="n">
-        <v>10573</v>
+        <v>10521</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
@@ -4734,10 +4986,10 @@
         </is>
       </c>
       <c r="F120" s="3" t="n">
-        <v>802</v>
+        <v>642</v>
       </c>
       <c r="G120" s="3" t="n">
-        <v>8636</v>
+        <v>6907</v>
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
@@ -4772,10 +5024,10 @@
         </is>
       </c>
       <c r="F121" s="3" t="n">
-        <v>1673</v>
+        <v>3414</v>
       </c>
       <c r="G121" s="3" t="n">
-        <v>18011</v>
+        <v>36752</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
@@ -4810,10 +5062,10 @@
         </is>
       </c>
       <c r="F122" s="3" t="n">
-        <v>624</v>
+        <v>463</v>
       </c>
       <c r="G122" s="3" t="n">
-        <v>6713</v>
+        <v>4985</v>
       </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
@@ -4886,10 +5138,10 @@
         </is>
       </c>
       <c r="F124" s="3" t="n">
-        <v>1340</v>
+        <v>692</v>
       </c>
       <c r="G124" s="3" t="n">
-        <v>14419</v>
+        <v>7451</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
@@ -4923,8 +5175,12 @@
           <t>J0H 1K0</t>
         </is>
       </c>
-      <c r="F125" s="3" t="n"/>
-      <c r="G125" s="3" t="n"/>
+      <c r="F125" s="3" t="n">
+        <v>374</v>
+      </c>
+      <c r="G125" s="3" t="n">
+        <v>4029</v>
+      </c>
       <c r="H125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
@@ -4954,10 +5210,10 @@
         </is>
       </c>
       <c r="F126" s="3" t="n">
-        <v>2221</v>
+        <v>665</v>
       </c>
       <c r="G126" s="3" t="n">
-        <v>23904</v>
+        <v>7153</v>
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
@@ -4992,10 +5248,10 @@
         </is>
       </c>
       <c r="F127" s="3" t="n">
-        <v>596</v>
+        <v>670</v>
       </c>
       <c r="G127" s="3" t="n">
-        <v>6412</v>
+        <v>7211</v>
       </c>
       <c r="H127" s="3" t="inlineStr">
         <is>
@@ -5030,10 +5286,10 @@
         </is>
       </c>
       <c r="F128" s="3" t="n">
-        <v>453</v>
+        <v>787</v>
       </c>
       <c r="G128" s="3" t="n">
-        <v>4871</v>
+        <v>8469</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
@@ -5068,10 +5324,10 @@
         </is>
       </c>
       <c r="F129" s="3" t="n">
-        <v>1873</v>
+        <v>1409</v>
       </c>
       <c r="G129" s="3" t="n">
-        <v>20158</v>
+        <v>15166</v>
       </c>
       <c r="H129" s="3" t="inlineStr">
         <is>
@@ -5182,10 +5438,10 @@
         </is>
       </c>
       <c r="F132" s="3" t="n">
-        <v>2646</v>
+        <v>3422</v>
       </c>
       <c r="G132" s="3" t="n">
-        <v>28485</v>
+        <v>36835</v>
       </c>
       <c r="H132" s="3" t="inlineStr">
         <is>
@@ -5296,10 +5552,10 @@
         </is>
       </c>
       <c r="F135" s="3" t="n">
-        <v>730</v>
+        <v>825</v>
       </c>
       <c r="G135" s="3" t="n">
-        <v>7854</v>
+        <v>8883</v>
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
@@ -5334,10 +5590,10 @@
         </is>
       </c>
       <c r="F136" s="3" t="n">
-        <v>1030</v>
+        <v>2867</v>
       </c>
       <c r="G136" s="3" t="n">
-        <v>11084</v>
+        <v>30857</v>
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
@@ -5410,10 +5666,10 @@
         </is>
       </c>
       <c r="F138" s="3" t="n">
-        <v>368</v>
+        <v>387</v>
       </c>
       <c r="G138" s="3" t="n">
-        <v>3962</v>
+        <v>4163</v>
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
@@ -5448,10 +5704,10 @@
         </is>
       </c>
       <c r="F139" s="3" t="n">
-        <v>109</v>
+        <v>745</v>
       </c>
       <c r="G139" s="3" t="n">
-        <v>1176</v>
+        <v>8020</v>
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
@@ -5524,10 +5780,10 @@
         </is>
       </c>
       <c r="F141" s="3" t="n">
-        <v>158</v>
+        <v>589</v>
       </c>
       <c r="G141" s="3" t="n">
-        <v>1701</v>
+        <v>6343</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
@@ -5600,10 +5856,10 @@
         </is>
       </c>
       <c r="F143" s="3" t="n">
-        <v>1203</v>
+        <v>574</v>
       </c>
       <c r="G143" s="3" t="n">
-        <v>12951</v>
+        <v>6175</v>
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
@@ -5638,10 +5894,10 @@
         </is>
       </c>
       <c r="F144" s="3" t="n">
-        <v>1400</v>
+        <v>1305</v>
       </c>
       <c r="G144" s="3" t="n">
-        <v>15069</v>
+        <v>14043</v>
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
@@ -5676,10 +5932,10 @@
         </is>
       </c>
       <c r="F145" s="3" t="n">
-        <v>1029</v>
+        <v>743</v>
       </c>
       <c r="G145" s="3" t="n">
-        <v>11077</v>
+        <v>8001</v>
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
@@ -5714,10 +5970,10 @@
         </is>
       </c>
       <c r="F146" s="3" t="n">
-        <v>68</v>
+        <v>760</v>
       </c>
       <c r="G146" s="3" t="n">
-        <v>732</v>
+        <v>8184</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
@@ -5752,10 +6008,10 @@
         </is>
       </c>
       <c r="F147" s="3" t="n">
-        <v>499</v>
+        <v>760</v>
       </c>
       <c r="G147" s="3" t="n">
-        <v>5373</v>
+        <v>8185</v>
       </c>
       <c r="H147" s="3" t="inlineStr">
         <is>
@@ -5790,10 +6046,10 @@
         </is>
       </c>
       <c r="F148" s="3" t="n">
-        <v>993</v>
+        <v>660</v>
       </c>
       <c r="G148" s="3" t="n">
-        <v>10687</v>
+        <v>7107</v>
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
@@ -5828,10 +6084,10 @@
         </is>
       </c>
       <c r="F149" s="3" t="n">
-        <v>402</v>
+        <v>506</v>
       </c>
       <c r="G149" s="3" t="n">
-        <v>4325</v>
+        <v>5445</v>
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
@@ -5904,10 +6160,10 @@
         </is>
       </c>
       <c r="F151" s="3" t="n">
-        <v>995</v>
+        <v>300</v>
       </c>
       <c r="G151" s="3" t="n">
-        <v>10710</v>
+        <v>3231</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
@@ -5942,10 +6198,10 @@
         </is>
       </c>
       <c r="F152" s="3" t="n">
-        <v>1925</v>
+        <v>988</v>
       </c>
       <c r="G152" s="3" t="n">
-        <v>20716</v>
+        <v>10636</v>
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
@@ -5980,10 +6236,10 @@
         </is>
       </c>
       <c r="F153" s="3" t="n">
-        <v>247</v>
+        <v>1160</v>
       </c>
       <c r="G153" s="3" t="n">
-        <v>2661</v>
+        <v>12485</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
@@ -6017,8 +6273,12 @@
           <t>J8C 2Z8</t>
         </is>
       </c>
-      <c r="F154" s="3" t="n"/>
-      <c r="G154" s="3" t="n"/>
+      <c r="F154" s="3" t="n">
+        <v>3722</v>
+      </c>
+      <c r="G154" s="3" t="n">
+        <v>40060</v>
+      </c>
       <c r="H154" s="3" t="inlineStr"/>
     </row>
     <row r="155">
@@ -6086,10 +6346,10 @@
         </is>
       </c>
       <c r="F156" s="3" t="n">
-        <v>2831</v>
+        <v>1410</v>
       </c>
       <c r="G156" s="3" t="n">
-        <v>30469</v>
+        <v>15172</v>
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
@@ -6124,10 +6384,10 @@
         </is>
       </c>
       <c r="F157" s="3" t="n">
-        <v>1430</v>
+        <v>1211</v>
       </c>
       <c r="G157" s="3" t="n">
-        <v>15393</v>
+        <v>13039</v>
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
@@ -6162,10 +6422,10 @@
         </is>
       </c>
       <c r="F158" s="3" t="n">
-        <v>1475</v>
+        <v>2649</v>
       </c>
       <c r="G158" s="3" t="n">
-        <v>15879</v>
+        <v>28519</v>
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
@@ -6200,10 +6460,10 @@
         </is>
       </c>
       <c r="F159" s="3" t="n">
-        <v>812</v>
+        <v>3124</v>
       </c>
       <c r="G159" s="3" t="n">
-        <v>8738</v>
+        <v>33623</v>
       </c>
       <c r="H159" s="3" t="inlineStr">
         <is>
@@ -6238,10 +6498,10 @@
         </is>
       </c>
       <c r="F160" s="3" t="n">
-        <v>757</v>
+        <v>746</v>
       </c>
       <c r="G160" s="3" t="n">
-        <v>8145</v>
+        <v>8032</v>
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
@@ -6276,10 +6536,10 @@
         </is>
       </c>
       <c r="F161" s="3" t="n">
-        <v>568</v>
+        <v>799</v>
       </c>
       <c r="G161" s="3" t="n">
-        <v>6114</v>
+        <v>8595</v>
       </c>
       <c r="H161" s="3" t="inlineStr">
         <is>
@@ -6428,10 +6688,10 @@
         </is>
       </c>
       <c r="F165" s="3" t="n">
-        <v>1211</v>
+        <v>1375</v>
       </c>
       <c r="G165" s="3" t="n">
-        <v>13039</v>
+        <v>14797</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
@@ -6465,8 +6725,12 @@
           <t>G0X 3G0</t>
         </is>
       </c>
-      <c r="F166" s="3" t="n"/>
-      <c r="G166" s="3" t="n"/>
+      <c r="F166" s="3" t="n">
+        <v>363</v>
+      </c>
+      <c r="G166" s="3" t="n">
+        <v>3903</v>
+      </c>
       <c r="H166" s="3" t="inlineStr"/>
     </row>
     <row r="167">
@@ -6496,10 +6760,10 @@
         </is>
       </c>
       <c r="F167" s="3" t="n">
-        <v>1224</v>
+        <v>1158</v>
       </c>
       <c r="G167" s="3" t="n">
-        <v>13171</v>
+        <v>12470</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
@@ -6534,10 +6798,10 @@
         </is>
       </c>
       <c r="F168" s="3" t="n">
-        <v>1402</v>
+        <v>1034</v>
       </c>
       <c r="G168" s="3" t="n">
-        <v>15095</v>
+        <v>11133</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
@@ -6610,10 +6874,10 @@
         </is>
       </c>
       <c r="F170" s="3" t="n">
-        <v>1071</v>
+        <v>1052</v>
       </c>
       <c r="G170" s="3" t="n">
-        <v>11526</v>
+        <v>11328</v>
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
@@ -6686,10 +6950,10 @@
         </is>
       </c>
       <c r="F172" s="3" t="n">
-        <v>1190</v>
+        <v>1600</v>
       </c>
       <c r="G172" s="3" t="n">
-        <v>12805</v>
+        <v>17228</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
@@ -6724,10 +6988,10 @@
         </is>
       </c>
       <c r="F173" s="3" t="n">
-        <v>1038</v>
+        <v>724</v>
       </c>
       <c r="G173" s="3" t="n">
-        <v>11174</v>
+        <v>7797</v>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
@@ -6762,10 +7026,10 @@
         </is>
       </c>
       <c r="F174" s="3" t="n">
-        <v>2471</v>
+        <v>762</v>
       </c>
       <c r="G174" s="3" t="n">
-        <v>26594</v>
+        <v>8198</v>
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
@@ -6800,10 +7064,10 @@
         </is>
       </c>
       <c r="F175" s="3" t="n">
-        <v>346</v>
+        <v>2474</v>
       </c>
       <c r="G175" s="3" t="n">
-        <v>3725</v>
+        <v>26628</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
@@ -6838,10 +7102,10 @@
         </is>
       </c>
       <c r="F176" s="3" t="n">
-        <v>151</v>
+        <v>789</v>
       </c>
       <c r="G176" s="3" t="n">
-        <v>1628</v>
+        <v>8489</v>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
@@ -6901,8 +7165,12 @@
       <c r="C178" s="3" t="inlineStr"/>
       <c r="D178" s="3" t="inlineStr"/>
       <c r="E178" s="3" t="inlineStr"/>
-      <c r="F178" s="3" t="n"/>
-      <c r="G178" s="3" t="n"/>
+      <c r="F178" s="3" t="n">
+        <v>481</v>
+      </c>
+      <c r="G178" s="3" t="n">
+        <v>5182</v>
+      </c>
       <c r="H178" s="3" t="inlineStr"/>
     </row>
     <row r="179">
@@ -6919,8 +7187,12 @@
       <c r="C179" s="3" t="inlineStr"/>
       <c r="D179" s="3" t="inlineStr"/>
       <c r="E179" s="3" t="inlineStr"/>
-      <c r="F179" s="3" t="n"/>
-      <c r="G179" s="3" t="n"/>
+      <c r="F179" s="3" t="n">
+        <v>2111</v>
+      </c>
+      <c r="G179" s="3" t="n">
+        <v>22723</v>
+      </c>
       <c r="H179" s="3" t="inlineStr"/>
     </row>
     <row r="180">
@@ -6937,8 +7209,12 @@
       <c r="C180" s="3" t="inlineStr"/>
       <c r="D180" s="3" t="inlineStr"/>
       <c r="E180" s="3" t="inlineStr"/>
-      <c r="F180" s="3" t="n"/>
-      <c r="G180" s="3" t="n"/>
+      <c r="F180" s="3" t="n">
+        <v>2083</v>
+      </c>
+      <c r="G180" s="3" t="n">
+        <v>22421</v>
+      </c>
       <c r="H180" s="3" t="inlineStr"/>
     </row>
     <row r="181">
@@ -6955,8 +7231,12 @@
       <c r="C181" s="3" t="inlineStr"/>
       <c r="D181" s="3" t="inlineStr"/>
       <c r="E181" s="3" t="inlineStr"/>
-      <c r="F181" s="3" t="n"/>
-      <c r="G181" s="3" t="n"/>
+      <c r="F181" s="3" t="n">
+        <v>3392</v>
+      </c>
+      <c r="G181" s="3" t="n">
+        <v>36512</v>
+      </c>
       <c r="H181" s="3" t="inlineStr"/>
     </row>
     <row r="182">
@@ -6973,8 +7253,12 @@
       <c r="C182" s="3" t="inlineStr"/>
       <c r="D182" s="3" t="inlineStr"/>
       <c r="E182" s="3" t="inlineStr"/>
-      <c r="F182" s="3" t="n"/>
-      <c r="G182" s="3" t="n"/>
+      <c r="F182" s="3" t="n">
+        <v>4714</v>
+      </c>
+      <c r="G182" s="3" t="n">
+        <v>50745</v>
+      </c>
       <c r="H182" s="3" t="inlineStr"/>
     </row>
     <row r="183">
@@ -6991,8 +7275,12 @@
       <c r="C183" s="3" t="inlineStr"/>
       <c r="D183" s="3" t="inlineStr"/>
       <c r="E183" s="3" t="inlineStr"/>
-      <c r="F183" s="3" t="n"/>
-      <c r="G183" s="3" t="n"/>
+      <c r="F183" s="3" t="n">
+        <v>4579</v>
+      </c>
+      <c r="G183" s="3" t="n">
+        <v>49287</v>
+      </c>
       <c r="H183" s="3" t="inlineStr"/>
     </row>
     <row r="184">
@@ -7009,8 +7297,12 @@
       <c r="C184" s="3" t="inlineStr"/>
       <c r="D184" s="3" t="inlineStr"/>
       <c r="E184" s="3" t="inlineStr"/>
-      <c r="F184" s="3" t="n"/>
-      <c r="G184" s="3" t="n"/>
+      <c r="F184" s="3" t="n">
+        <v>2442</v>
+      </c>
+      <c r="G184" s="3" t="n">
+        <v>26280</v>
+      </c>
       <c r="H184" s="3" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add domain testing script and DNS verification results
Adds test_domaines.py: a standalone script that checks A/MX DNS
records and HTTP response (parking-page detection) to classify a
domain as an active site, mail-only, or dead. Ran the DNS-only
portion here (HTTP is blocked by sandbox egress policy) and found
3 of 36 domains have no DNS records at all, meaning they were
likely misidentified by the earlier research pass. New "DNS (A/MX)"
column records the finding per row.
</commit_message>
<xml_diff>
--- a/BMR_prospection.xlsx
+++ b/BMR_prospection.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P186"/>
+  <dimension ref="A1:Q186"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" style="4" min="1" max="1"/>
@@ -465,6 +465,7 @@
     <col width="24.33203125" bestFit="1" customWidth="1" style="4" min="14" max="14"/>
     <col width="25" bestFit="1" customWidth="1" style="4" min="15" max="15"/>
     <col width="14" customWidth="1" style="4" min="16" max="16384"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,6 +549,11 @@
           <t>Statut domaine</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>DNS (A/MX)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1723,6 +1729,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q20" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1832,6 +1843,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q22" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1891,6 +1907,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q23" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -2055,6 +2076,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q26" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -2114,6 +2140,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q27" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -2173,6 +2204,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q28" s="17" t="inlineStr">
+        <is>
+          <t>A seul</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -2232,6 +2268,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q29" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2391,6 +2432,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q32" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2450,6 +2496,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q33" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2619,6 +2670,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q36" s="17" t="inlineStr">
+        <is>
+          <t>AUCUN</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2678,6 +2734,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q37" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2787,6 +2848,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q39" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2846,6 +2912,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q40" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2905,6 +2976,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q41" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2964,6 +3040,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q42" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -3023,6 +3104,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q43" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -3082,6 +3168,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q44" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -3141,6 +3232,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q45" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -3200,6 +3296,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q46" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -3259,6 +3360,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q47" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3368,6 +3474,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q49" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3477,6 +3588,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q51" s="17" t="inlineStr">
+        <is>
+          <t>A seul</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -3591,6 +3707,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q53" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -3650,6 +3771,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q54" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -3709,6 +3835,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q55" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -3768,6 +3899,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q56" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3877,6 +4013,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q58" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -3936,6 +4077,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q59" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -3995,6 +4141,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q60" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4104,6 +4255,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q62" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -4163,6 +4319,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q63" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4532,6 +4693,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q70" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4641,6 +4807,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q72" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -4755,6 +4926,11 @@
           <t>Inactif</t>
         </is>
       </c>
+      <c r="Q74" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -4814,6 +4990,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q75" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -4873,6 +5054,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q76" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -4932,6 +5118,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q77" s="17" t="inlineStr">
+        <is>
+          <t>AUCUN</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5256,6 +5447,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q83" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -5315,6 +5511,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q84" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -5479,6 +5680,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q87" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5588,6 +5794,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q89" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -5647,6 +5858,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q90" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5756,6 +5972,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q92" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5920,6 +6141,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q95" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6134,6 +6360,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q99" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -6246,6 +6477,11 @@
       <c r="P101" s="17" t="inlineStr">
         <is>
           <t>Opérationnel</t>
+        </is>
+      </c>
+      <c r="Q101" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
         </is>
       </c>
     </row>
@@ -6308,6 +6544,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q102" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -6422,6 +6663,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q104" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -6481,6 +6727,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q105" s="17" t="inlineStr">
+        <is>
+          <t>A seul</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6919,6 +7170,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q113" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
@@ -6978,6 +7234,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q114" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -7037,6 +7298,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q115" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
@@ -7151,6 +7417,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q117" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
@@ -7210,6 +7481,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q118" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -7324,6 +7600,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q120" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -7383,6 +7664,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q121" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -7552,6 +7838,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q124" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -7826,6 +8117,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q129" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
@@ -7885,6 +8181,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q130" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -7999,6 +8300,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q132" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -8058,6 +8364,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q133" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8387,6 +8698,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q139" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
@@ -8556,6 +8872,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q142" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -8830,6 +9151,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q147" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
@@ -8889,6 +9215,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q148" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -9003,6 +9334,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q150" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -9062,6 +9398,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q151" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
@@ -9121,6 +9462,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q152" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -9180,6 +9526,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q153" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
@@ -9292,6 +9643,11 @@
       <c r="P155" s="17" t="inlineStr">
         <is>
           <t>Opérationnel</t>
+        </is>
+      </c>
+      <c r="Q155" s="17" t="inlineStr">
+        <is>
+          <t>AUCUN</t>
         </is>
       </c>
     </row>
@@ -9669,6 +10025,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q162" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -9728,6 +10089,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q163" s="17" t="inlineStr">
+        <is>
+          <t>A seul</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
@@ -9787,6 +10153,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q164" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -9956,6 +10327,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q167" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
@@ -10070,6 +10446,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q169" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
@@ -10129,6 +10510,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q170" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -10188,6 +10574,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q171" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
@@ -10462,6 +10853,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q176" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -10631,6 +11027,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q179" s="17" t="inlineStr">
+        <is>
+          <t>A seul</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
@@ -10690,6 +11091,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q180" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -10749,6 +11155,11 @@
           <t>Opérationnel</t>
         </is>
       </c>
+      <c r="Q181" s="17" t="inlineStr">
+        <is>
+          <t>A+MX</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
@@ -10916,6 +11327,11 @@
       <c r="P184" s="17" t="inlineStr">
         <is>
           <t>Opérationnel</t>
+        </is>
+      </c>
+      <c r="Q184" s="17" t="inlineStr">
+        <is>
+          <t>A seul</t>
         </is>
       </c>
     </row>

</xml_diff>